<commit_message>
Split discovery and application sources
</commit_message>
<xml_diff>
--- a/templates/linc_tracker_template.xlsx
+++ b/templates/linc_tracker_template.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" r:id="R2b751889b2644c32"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Input" sheetId="2" r:id="Rd0bd20791d504fc9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Applications" sheetId="3" r:id="Rcea2739aa7c342e1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" r:id="Ra57c4482805a49f8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Input" sheetId="2" r:id="Rf98d8f696cda4a2c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Applications" sheetId="3" r:id="R2d9c78b21d994128"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -59,7 +59,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="5">
+  <x:fills count="6">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -79,6 +79,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFFF8F4"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFC95335"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -185,7 +190,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="44">
+  <x:cellXfs count="49">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -269,6 +274,17 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -360,8 +376,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ApplicationsTable" displayName="ApplicationsTable" ref="A1:J201" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="10">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ApplicationsTable" displayName="ApplicationsTable" ref="A1:K201" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="11">
     <x:tableColumn id="1" name="Date Applied"/>
     <x:tableColumn id="2" name="Company"/>
     <x:tableColumn id="3" name="Job Title"/>
@@ -371,7 +387,8 @@
     <x:tableColumn id="7" name="Work Type"/>
     <x:tableColumn id="8" name="Salary Range"/>
     <x:tableColumn id="9" name="Follow-up"/>
-    <x:tableColumn id="10" name="Source"/>
+    <x:tableColumn id="10" name="Found On"/>
+    <x:tableColumn id="11" name="Application Portal"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium3" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -612,7 +629,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B5" s="24" t="str">
-        <x:v>Run Linc to fill in the job details.</x:v>
+        <x:v>Choose where you found the jobs in Linc, or leave Auto to use clues in the link.</x:v>
       </x:c>
       <x:c r="C5" s="25" t="str"/>
       <x:c r="D5" s="25" t="str"/>
@@ -624,7 +641,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B6" s="24" t="str">
-        <x:v>Check every row marked Review or Error before saving it.</x:v>
+        <x:v>Linc detects the application portal from each URL and fills in the job details.</x:v>
       </x:c>
       <x:c r="C6" s="25" t="str"/>
       <x:c r="D6" s="25" t="str"/>
@@ -636,7 +653,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B7" s="24" t="str">
-        <x:v>Finished jobs appear on the Applications sheet.</x:v>
+        <x:v>Check rows marked Review or Error before adding finished jobs to Applications.</x:v>
       </x:c>
       <x:c r="C7" s="25" t="str"/>
       <x:c r="D7" s="25" t="str"/>
@@ -681,7 +698,7 @@
         <x:v>Job Link</x:v>
       </x:c>
       <x:c r="B1" s="32" t="str">
-        <x:v>Source</x:v>
+        <x:v>Found On</x:v>
       </x:c>
       <x:c r="C1" s="32" t="str">
         <x:v>Notes</x:v>
@@ -2344,7 +2361,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R62d9e52fe07049d7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd10f70f5f9a04449"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2362,7 +2379,8 @@
     <x:col min="7" max="7" width="16" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="22" hidden="0" customWidth="1"/>
     <x:col min="9" max="9" width="14" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="18" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="20" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="22" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
@@ -2394,7 +2412,10 @@
         <x:v>Follow-up</x:v>
       </x:c>
       <x:c r="J1" s="32" t="str">
-        <x:v>Source</x:v>
+        <x:v>Found On</x:v>
+      </x:c>
+      <x:c r="K1" s="48" t="str">
+        <x:v>Application Portal</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
@@ -2408,6 +2429,7 @@
       <x:c r="H2" s="36"/>
       <x:c r="I2" s="39"/>
       <x:c r="J2" s="37"/>
+      <x:c r="K2"/>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="39"/>
@@ -2420,6 +2442,7 @@
       <x:c r="H3" s="36"/>
       <x:c r="I3" s="39"/>
       <x:c r="J3" s="37"/>
+      <x:c r="K3"/>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="39"/>
@@ -2432,6 +2455,7 @@
       <x:c r="H4" s="36"/>
       <x:c r="I4" s="39"/>
       <x:c r="J4" s="37"/>
+      <x:c r="K4"/>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="39"/>
@@ -2444,6 +2468,7 @@
       <x:c r="H5" s="36"/>
       <x:c r="I5" s="39"/>
       <x:c r="J5" s="37"/>
+      <x:c r="K5"/>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="39"/>
@@ -2456,6 +2481,7 @@
       <x:c r="H6" s="36"/>
       <x:c r="I6" s="39"/>
       <x:c r="J6" s="37"/>
+      <x:c r="K6"/>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="39"/>
@@ -2468,6 +2494,7 @@
       <x:c r="H7" s="36"/>
       <x:c r="I7" s="39"/>
       <x:c r="J7" s="37"/>
+      <x:c r="K7"/>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="39"/>
@@ -2480,6 +2507,7 @@
       <x:c r="H8" s="36"/>
       <x:c r="I8" s="39"/>
       <x:c r="J8" s="37"/>
+      <x:c r="K8"/>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="39"/>
@@ -2492,6 +2520,7 @@
       <x:c r="H9" s="36"/>
       <x:c r="I9" s="39"/>
       <x:c r="J9" s="37"/>
+      <x:c r="K9"/>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="39"/>
@@ -2504,6 +2533,7 @@
       <x:c r="H10" s="36"/>
       <x:c r="I10" s="39"/>
       <x:c r="J10" s="37"/>
+      <x:c r="K10"/>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="39"/>
@@ -2516,6 +2546,7 @@
       <x:c r="H11" s="36"/>
       <x:c r="I11" s="39"/>
       <x:c r="J11" s="37"/>
+      <x:c r="K11"/>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="39"/>
@@ -2528,6 +2559,7 @@
       <x:c r="H12" s="36"/>
       <x:c r="I12" s="39"/>
       <x:c r="J12" s="37"/>
+      <x:c r="K12"/>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="39"/>
@@ -2540,6 +2572,7 @@
       <x:c r="H13" s="36"/>
       <x:c r="I13" s="39"/>
       <x:c r="J13" s="37"/>
+      <x:c r="K13"/>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="39"/>
@@ -2552,6 +2585,7 @@
       <x:c r="H14" s="36"/>
       <x:c r="I14" s="39"/>
       <x:c r="J14" s="37"/>
+      <x:c r="K14"/>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="39"/>
@@ -2564,6 +2598,7 @@
       <x:c r="H15" s="36"/>
       <x:c r="I15" s="39"/>
       <x:c r="J15" s="37"/>
+      <x:c r="K15"/>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="39"/>
@@ -2576,6 +2611,7 @@
       <x:c r="H16" s="36"/>
       <x:c r="I16" s="39"/>
       <x:c r="J16" s="37"/>
+      <x:c r="K16"/>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="39"/>
@@ -2588,6 +2624,7 @@
       <x:c r="H17" s="36"/>
       <x:c r="I17" s="39"/>
       <x:c r="J17" s="37"/>
+      <x:c r="K17"/>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="39"/>
@@ -2600,6 +2637,7 @@
       <x:c r="H18" s="36"/>
       <x:c r="I18" s="39"/>
       <x:c r="J18" s="37"/>
+      <x:c r="K18"/>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="39"/>
@@ -2612,6 +2650,7 @@
       <x:c r="H19" s="36"/>
       <x:c r="I19" s="39"/>
       <x:c r="J19" s="37"/>
+      <x:c r="K19"/>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="39"/>
@@ -2624,6 +2663,7 @@
       <x:c r="H20" s="36"/>
       <x:c r="I20" s="39"/>
       <x:c r="J20" s="37"/>
+      <x:c r="K20"/>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="39"/>
@@ -2636,6 +2676,7 @@
       <x:c r="H21" s="36"/>
       <x:c r="I21" s="39"/>
       <x:c r="J21" s="37"/>
+      <x:c r="K21"/>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="39"/>
@@ -2648,6 +2689,7 @@
       <x:c r="H22" s="36"/>
       <x:c r="I22" s="39"/>
       <x:c r="J22" s="37"/>
+      <x:c r="K22"/>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="39"/>
@@ -2660,6 +2702,7 @@
       <x:c r="H23" s="36"/>
       <x:c r="I23" s="39"/>
       <x:c r="J23" s="37"/>
+      <x:c r="K23"/>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="39"/>
@@ -2672,6 +2715,7 @@
       <x:c r="H24" s="36"/>
       <x:c r="I24" s="39"/>
       <x:c r="J24" s="37"/>
+      <x:c r="K24"/>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="39"/>
@@ -2684,6 +2728,7 @@
       <x:c r="H25" s="36"/>
       <x:c r="I25" s="39"/>
       <x:c r="J25" s="37"/>
+      <x:c r="K25"/>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="39"/>
@@ -2696,6 +2741,7 @@
       <x:c r="H26" s="36"/>
       <x:c r="I26" s="39"/>
       <x:c r="J26" s="37"/>
+      <x:c r="K26"/>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="39"/>
@@ -2708,6 +2754,7 @@
       <x:c r="H27" s="36"/>
       <x:c r="I27" s="39"/>
       <x:c r="J27" s="37"/>
+      <x:c r="K27"/>
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="39"/>
@@ -2720,6 +2767,7 @@
       <x:c r="H28" s="36"/>
       <x:c r="I28" s="39"/>
       <x:c r="J28" s="37"/>
+      <x:c r="K28"/>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="39"/>
@@ -2732,6 +2780,7 @@
       <x:c r="H29" s="36"/>
       <x:c r="I29" s="39"/>
       <x:c r="J29" s="37"/>
+      <x:c r="K29"/>
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="39"/>
@@ -2744,6 +2793,7 @@
       <x:c r="H30" s="36"/>
       <x:c r="I30" s="39"/>
       <x:c r="J30" s="37"/>
+      <x:c r="K30"/>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="39"/>
@@ -2756,6 +2806,7 @@
       <x:c r="H31" s="36"/>
       <x:c r="I31" s="39"/>
       <x:c r="J31" s="37"/>
+      <x:c r="K31"/>
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="39"/>
@@ -2768,6 +2819,7 @@
       <x:c r="H32" s="36"/>
       <x:c r="I32" s="39"/>
       <x:c r="J32" s="37"/>
+      <x:c r="K32"/>
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="39"/>
@@ -2780,6 +2832,7 @@
       <x:c r="H33" s="36"/>
       <x:c r="I33" s="39"/>
       <x:c r="J33" s="37"/>
+      <x:c r="K33"/>
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="39"/>
@@ -2792,6 +2845,7 @@
       <x:c r="H34" s="36"/>
       <x:c r="I34" s="39"/>
       <x:c r="J34" s="37"/>
+      <x:c r="K34"/>
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="39"/>
@@ -2804,6 +2858,7 @@
       <x:c r="H35" s="36"/>
       <x:c r="I35" s="39"/>
       <x:c r="J35" s="37"/>
+      <x:c r="K35"/>
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="39"/>
@@ -2816,6 +2871,7 @@
       <x:c r="H36" s="36"/>
       <x:c r="I36" s="39"/>
       <x:c r="J36" s="37"/>
+      <x:c r="K36"/>
     </x:row>
     <x:row r="37">
       <x:c r="A37" s="39"/>
@@ -2828,6 +2884,7 @@
       <x:c r="H37" s="36"/>
       <x:c r="I37" s="39"/>
       <x:c r="J37" s="37"/>
+      <x:c r="K37"/>
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="39"/>
@@ -2840,6 +2897,7 @@
       <x:c r="H38" s="36"/>
       <x:c r="I38" s="39"/>
       <x:c r="J38" s="37"/>
+      <x:c r="K38"/>
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="39"/>
@@ -2852,6 +2910,7 @@
       <x:c r="H39" s="36"/>
       <x:c r="I39" s="39"/>
       <x:c r="J39" s="37"/>
+      <x:c r="K39"/>
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="39"/>
@@ -2864,6 +2923,7 @@
       <x:c r="H40" s="36"/>
       <x:c r="I40" s="39"/>
       <x:c r="J40" s="37"/>
+      <x:c r="K40"/>
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="39"/>
@@ -2876,6 +2936,7 @@
       <x:c r="H41" s="36"/>
       <x:c r="I41" s="39"/>
       <x:c r="J41" s="37"/>
+      <x:c r="K41"/>
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="39"/>
@@ -2888,6 +2949,7 @@
       <x:c r="H42" s="36"/>
       <x:c r="I42" s="39"/>
       <x:c r="J42" s="37"/>
+      <x:c r="K42"/>
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="39"/>
@@ -2900,6 +2962,7 @@
       <x:c r="H43" s="36"/>
       <x:c r="I43" s="39"/>
       <x:c r="J43" s="37"/>
+      <x:c r="K43"/>
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="39"/>
@@ -2912,6 +2975,7 @@
       <x:c r="H44" s="36"/>
       <x:c r="I44" s="39"/>
       <x:c r="J44" s="37"/>
+      <x:c r="K44"/>
     </x:row>
     <x:row r="45">
       <x:c r="A45" s="39"/>
@@ -2924,6 +2988,7 @@
       <x:c r="H45" s="36"/>
       <x:c r="I45" s="39"/>
       <x:c r="J45" s="37"/>
+      <x:c r="K45"/>
     </x:row>
     <x:row r="46">
       <x:c r="A46" s="39"/>
@@ -2936,6 +3001,7 @@
       <x:c r="H46" s="36"/>
       <x:c r="I46" s="39"/>
       <x:c r="J46" s="37"/>
+      <x:c r="K46"/>
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="39"/>
@@ -2948,6 +3014,7 @@
       <x:c r="H47" s="36"/>
       <x:c r="I47" s="39"/>
       <x:c r="J47" s="37"/>
+      <x:c r="K47"/>
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="39"/>
@@ -2960,6 +3027,7 @@
       <x:c r="H48" s="36"/>
       <x:c r="I48" s="39"/>
       <x:c r="J48" s="37"/>
+      <x:c r="K48"/>
     </x:row>
     <x:row r="49">
       <x:c r="A49" s="39"/>
@@ -2972,6 +3040,7 @@
       <x:c r="H49" s="36"/>
       <x:c r="I49" s="39"/>
       <x:c r="J49" s="37"/>
+      <x:c r="K49"/>
     </x:row>
     <x:row r="50">
       <x:c r="A50" s="39"/>
@@ -2984,6 +3053,7 @@
       <x:c r="H50" s="36"/>
       <x:c r="I50" s="39"/>
       <x:c r="J50" s="37"/>
+      <x:c r="K50"/>
     </x:row>
     <x:row r="51">
       <x:c r="A51" s="39"/>
@@ -2996,6 +3066,7 @@
       <x:c r="H51" s="36"/>
       <x:c r="I51" s="39"/>
       <x:c r="J51" s="37"/>
+      <x:c r="K51"/>
     </x:row>
     <x:row r="52">
       <x:c r="A52" s="39"/>
@@ -3008,6 +3079,7 @@
       <x:c r="H52" s="36"/>
       <x:c r="I52" s="39"/>
       <x:c r="J52" s="37"/>
+      <x:c r="K52"/>
     </x:row>
     <x:row r="53">
       <x:c r="A53" s="39"/>
@@ -3020,6 +3092,7 @@
       <x:c r="H53" s="36"/>
       <x:c r="I53" s="39"/>
       <x:c r="J53" s="37"/>
+      <x:c r="K53"/>
     </x:row>
     <x:row r="54">
       <x:c r="A54" s="39"/>
@@ -3032,6 +3105,7 @@
       <x:c r="H54" s="36"/>
       <x:c r="I54" s="39"/>
       <x:c r="J54" s="37"/>
+      <x:c r="K54"/>
     </x:row>
     <x:row r="55">
       <x:c r="A55" s="39"/>
@@ -3044,6 +3118,7 @@
       <x:c r="H55" s="36"/>
       <x:c r="I55" s="39"/>
       <x:c r="J55" s="37"/>
+      <x:c r="K55"/>
     </x:row>
     <x:row r="56">
       <x:c r="A56" s="39"/>
@@ -3056,6 +3131,7 @@
       <x:c r="H56" s="36"/>
       <x:c r="I56" s="39"/>
       <x:c r="J56" s="37"/>
+      <x:c r="K56"/>
     </x:row>
     <x:row r="57">
       <x:c r="A57" s="39"/>
@@ -3068,6 +3144,7 @@
       <x:c r="H57" s="36"/>
       <x:c r="I57" s="39"/>
       <x:c r="J57" s="37"/>
+      <x:c r="K57"/>
     </x:row>
     <x:row r="58">
       <x:c r="A58" s="39"/>
@@ -3080,6 +3157,7 @@
       <x:c r="H58" s="36"/>
       <x:c r="I58" s="39"/>
       <x:c r="J58" s="37"/>
+      <x:c r="K58"/>
     </x:row>
     <x:row r="59">
       <x:c r="A59" s="39"/>
@@ -3092,6 +3170,7 @@
       <x:c r="H59" s="36"/>
       <x:c r="I59" s="39"/>
       <x:c r="J59" s="37"/>
+      <x:c r="K59"/>
     </x:row>
     <x:row r="60">
       <x:c r="A60" s="39"/>
@@ -3104,6 +3183,7 @@
       <x:c r="H60" s="36"/>
       <x:c r="I60" s="39"/>
       <x:c r="J60" s="37"/>
+      <x:c r="K60"/>
     </x:row>
     <x:row r="61">
       <x:c r="A61" s="39"/>
@@ -3116,6 +3196,7 @@
       <x:c r="H61" s="36"/>
       <x:c r="I61" s="39"/>
       <x:c r="J61" s="37"/>
+      <x:c r="K61"/>
     </x:row>
     <x:row r="62">
       <x:c r="A62" s="39"/>
@@ -3128,6 +3209,7 @@
       <x:c r="H62" s="36"/>
       <x:c r="I62" s="39"/>
       <x:c r="J62" s="37"/>
+      <x:c r="K62"/>
     </x:row>
     <x:row r="63">
       <x:c r="A63" s="39"/>
@@ -3140,6 +3222,7 @@
       <x:c r="H63" s="36"/>
       <x:c r="I63" s="39"/>
       <x:c r="J63" s="37"/>
+      <x:c r="K63"/>
     </x:row>
     <x:row r="64">
       <x:c r="A64" s="39"/>
@@ -3152,6 +3235,7 @@
       <x:c r="H64" s="36"/>
       <x:c r="I64" s="39"/>
       <x:c r="J64" s="37"/>
+      <x:c r="K64"/>
     </x:row>
     <x:row r="65">
       <x:c r="A65" s="39"/>
@@ -3164,6 +3248,7 @@
       <x:c r="H65" s="36"/>
       <x:c r="I65" s="39"/>
       <x:c r="J65" s="37"/>
+      <x:c r="K65"/>
     </x:row>
     <x:row r="66">
       <x:c r="A66" s="39"/>
@@ -3176,6 +3261,7 @@
       <x:c r="H66" s="36"/>
       <x:c r="I66" s="39"/>
       <x:c r="J66" s="37"/>
+      <x:c r="K66"/>
     </x:row>
     <x:row r="67">
       <x:c r="A67" s="39"/>
@@ -3188,6 +3274,7 @@
       <x:c r="H67" s="36"/>
       <x:c r="I67" s="39"/>
       <x:c r="J67" s="37"/>
+      <x:c r="K67"/>
     </x:row>
     <x:row r="68">
       <x:c r="A68" s="39"/>
@@ -3200,6 +3287,7 @@
       <x:c r="H68" s="36"/>
       <x:c r="I68" s="39"/>
       <x:c r="J68" s="37"/>
+      <x:c r="K68"/>
     </x:row>
     <x:row r="69">
       <x:c r="A69" s="39"/>
@@ -3212,6 +3300,7 @@
       <x:c r="H69" s="36"/>
       <x:c r="I69" s="39"/>
       <x:c r="J69" s="37"/>
+      <x:c r="K69"/>
     </x:row>
     <x:row r="70">
       <x:c r="A70" s="39"/>
@@ -3224,6 +3313,7 @@
       <x:c r="H70" s="36"/>
       <x:c r="I70" s="39"/>
       <x:c r="J70" s="37"/>
+      <x:c r="K70"/>
     </x:row>
     <x:row r="71">
       <x:c r="A71" s="39"/>
@@ -3236,6 +3326,7 @@
       <x:c r="H71" s="36"/>
       <x:c r="I71" s="39"/>
       <x:c r="J71" s="37"/>
+      <x:c r="K71"/>
     </x:row>
     <x:row r="72">
       <x:c r="A72" s="39"/>
@@ -3248,6 +3339,7 @@
       <x:c r="H72" s="36"/>
       <x:c r="I72" s="39"/>
       <x:c r="J72" s="37"/>
+      <x:c r="K72"/>
     </x:row>
     <x:row r="73">
       <x:c r="A73" s="39"/>
@@ -3260,6 +3352,7 @@
       <x:c r="H73" s="36"/>
       <x:c r="I73" s="39"/>
       <x:c r="J73" s="37"/>
+      <x:c r="K73"/>
     </x:row>
     <x:row r="74">
       <x:c r="A74" s="39"/>
@@ -3272,6 +3365,7 @@
       <x:c r="H74" s="36"/>
       <x:c r="I74" s="39"/>
       <x:c r="J74" s="37"/>
+      <x:c r="K74"/>
     </x:row>
     <x:row r="75">
       <x:c r="A75" s="39"/>
@@ -3284,6 +3378,7 @@
       <x:c r="H75" s="36"/>
       <x:c r="I75" s="39"/>
       <x:c r="J75" s="37"/>
+      <x:c r="K75"/>
     </x:row>
     <x:row r="76">
       <x:c r="A76" s="39"/>
@@ -3296,6 +3391,7 @@
       <x:c r="H76" s="36"/>
       <x:c r="I76" s="39"/>
       <x:c r="J76" s="37"/>
+      <x:c r="K76"/>
     </x:row>
     <x:row r="77">
       <x:c r="A77" s="39"/>
@@ -3308,6 +3404,7 @@
       <x:c r="H77" s="36"/>
       <x:c r="I77" s="39"/>
       <x:c r="J77" s="37"/>
+      <x:c r="K77"/>
     </x:row>
     <x:row r="78">
       <x:c r="A78" s="39"/>
@@ -3320,6 +3417,7 @@
       <x:c r="H78" s="36"/>
       <x:c r="I78" s="39"/>
       <x:c r="J78" s="37"/>
+      <x:c r="K78"/>
     </x:row>
     <x:row r="79">
       <x:c r="A79" s="39"/>
@@ -3332,6 +3430,7 @@
       <x:c r="H79" s="36"/>
       <x:c r="I79" s="39"/>
       <x:c r="J79" s="37"/>
+      <x:c r="K79"/>
     </x:row>
     <x:row r="80">
       <x:c r="A80" s="39"/>
@@ -3344,6 +3443,7 @@
       <x:c r="H80" s="36"/>
       <x:c r="I80" s="39"/>
       <x:c r="J80" s="37"/>
+      <x:c r="K80"/>
     </x:row>
     <x:row r="81">
       <x:c r="A81" s="39"/>
@@ -3356,6 +3456,7 @@
       <x:c r="H81" s="36"/>
       <x:c r="I81" s="39"/>
       <x:c r="J81" s="37"/>
+      <x:c r="K81"/>
     </x:row>
     <x:row r="82">
       <x:c r="A82" s="39"/>
@@ -3368,6 +3469,7 @@
       <x:c r="H82" s="36"/>
       <x:c r="I82" s="39"/>
       <x:c r="J82" s="37"/>
+      <x:c r="K82"/>
     </x:row>
     <x:row r="83">
       <x:c r="A83" s="39"/>
@@ -3380,6 +3482,7 @@
       <x:c r="H83" s="36"/>
       <x:c r="I83" s="39"/>
       <x:c r="J83" s="37"/>
+      <x:c r="K83"/>
     </x:row>
     <x:row r="84">
       <x:c r="A84" s="39"/>
@@ -3392,6 +3495,7 @@
       <x:c r="H84" s="36"/>
       <x:c r="I84" s="39"/>
       <x:c r="J84" s="37"/>
+      <x:c r="K84"/>
     </x:row>
     <x:row r="85">
       <x:c r="A85" s="39"/>
@@ -3404,6 +3508,7 @@
       <x:c r="H85" s="36"/>
       <x:c r="I85" s="39"/>
       <x:c r="J85" s="37"/>
+      <x:c r="K85"/>
     </x:row>
     <x:row r="86">
       <x:c r="A86" s="39"/>
@@ -3416,6 +3521,7 @@
       <x:c r="H86" s="36"/>
       <x:c r="I86" s="39"/>
       <x:c r="J86" s="37"/>
+      <x:c r="K86"/>
     </x:row>
     <x:row r="87">
       <x:c r="A87" s="39"/>
@@ -3428,6 +3534,7 @@
       <x:c r="H87" s="36"/>
       <x:c r="I87" s="39"/>
       <x:c r="J87" s="37"/>
+      <x:c r="K87"/>
     </x:row>
     <x:row r="88">
       <x:c r="A88" s="39"/>
@@ -3440,6 +3547,7 @@
       <x:c r="H88" s="36"/>
       <x:c r="I88" s="39"/>
       <x:c r="J88" s="37"/>
+      <x:c r="K88"/>
     </x:row>
     <x:row r="89">
       <x:c r="A89" s="39"/>
@@ -3452,6 +3560,7 @@
       <x:c r="H89" s="36"/>
       <x:c r="I89" s="39"/>
       <x:c r="J89" s="37"/>
+      <x:c r="K89"/>
     </x:row>
     <x:row r="90">
       <x:c r="A90" s="39"/>
@@ -3464,6 +3573,7 @@
       <x:c r="H90" s="36"/>
       <x:c r="I90" s="39"/>
       <x:c r="J90" s="37"/>
+      <x:c r="K90"/>
     </x:row>
     <x:row r="91">
       <x:c r="A91" s="39"/>
@@ -3476,6 +3586,7 @@
       <x:c r="H91" s="36"/>
       <x:c r="I91" s="39"/>
       <x:c r="J91" s="37"/>
+      <x:c r="K91"/>
     </x:row>
     <x:row r="92">
       <x:c r="A92" s="39"/>
@@ -3488,6 +3599,7 @@
       <x:c r="H92" s="36"/>
       <x:c r="I92" s="39"/>
       <x:c r="J92" s="37"/>
+      <x:c r="K92"/>
     </x:row>
     <x:row r="93">
       <x:c r="A93" s="39"/>
@@ -3500,6 +3612,7 @@
       <x:c r="H93" s="36"/>
       <x:c r="I93" s="39"/>
       <x:c r="J93" s="37"/>
+      <x:c r="K93"/>
     </x:row>
     <x:row r="94">
       <x:c r="A94" s="39"/>
@@ -3512,6 +3625,7 @@
       <x:c r="H94" s="36"/>
       <x:c r="I94" s="39"/>
       <x:c r="J94" s="37"/>
+      <x:c r="K94"/>
     </x:row>
     <x:row r="95">
       <x:c r="A95" s="39"/>
@@ -3524,6 +3638,7 @@
       <x:c r="H95" s="36"/>
       <x:c r="I95" s="39"/>
       <x:c r="J95" s="37"/>
+      <x:c r="K95"/>
     </x:row>
     <x:row r="96">
       <x:c r="A96" s="39"/>
@@ -3536,6 +3651,7 @@
       <x:c r="H96" s="36"/>
       <x:c r="I96" s="39"/>
       <x:c r="J96" s="37"/>
+      <x:c r="K96"/>
     </x:row>
     <x:row r="97">
       <x:c r="A97" s="39"/>
@@ -3548,6 +3664,7 @@
       <x:c r="H97" s="36"/>
       <x:c r="I97" s="39"/>
       <x:c r="J97" s="37"/>
+      <x:c r="K97"/>
     </x:row>
     <x:row r="98">
       <x:c r="A98" s="39"/>
@@ -3560,6 +3677,7 @@
       <x:c r="H98" s="36"/>
       <x:c r="I98" s="39"/>
       <x:c r="J98" s="37"/>
+      <x:c r="K98"/>
     </x:row>
     <x:row r="99">
       <x:c r="A99" s="39"/>
@@ -3572,6 +3690,7 @@
       <x:c r="H99" s="36"/>
       <x:c r="I99" s="39"/>
       <x:c r="J99" s="37"/>
+      <x:c r="K99"/>
     </x:row>
     <x:row r="100">
       <x:c r="A100" s="39"/>
@@ -3584,6 +3703,7 @@
       <x:c r="H100" s="36"/>
       <x:c r="I100" s="39"/>
       <x:c r="J100" s="37"/>
+      <x:c r="K100"/>
     </x:row>
     <x:row r="101">
       <x:c r="A101" s="39"/>
@@ -3596,6 +3716,7 @@
       <x:c r="H101" s="36"/>
       <x:c r="I101" s="39"/>
       <x:c r="J101" s="37"/>
+      <x:c r="K101"/>
     </x:row>
     <x:row r="102">
       <x:c r="A102" s="39"/>
@@ -3608,6 +3729,7 @@
       <x:c r="H102" s="36"/>
       <x:c r="I102" s="39"/>
       <x:c r="J102" s="37"/>
+      <x:c r="K102"/>
     </x:row>
     <x:row r="103">
       <x:c r="A103" s="39"/>
@@ -3620,6 +3742,7 @@
       <x:c r="H103" s="36"/>
       <x:c r="I103" s="39"/>
       <x:c r="J103" s="37"/>
+      <x:c r="K103"/>
     </x:row>
     <x:row r="104">
       <x:c r="A104" s="39"/>
@@ -3632,6 +3755,7 @@
       <x:c r="H104" s="36"/>
       <x:c r="I104" s="39"/>
       <x:c r="J104" s="37"/>
+      <x:c r="K104"/>
     </x:row>
     <x:row r="105">
       <x:c r="A105" s="39"/>
@@ -3644,6 +3768,7 @@
       <x:c r="H105" s="36"/>
       <x:c r="I105" s="39"/>
       <x:c r="J105" s="37"/>
+      <x:c r="K105"/>
     </x:row>
     <x:row r="106">
       <x:c r="A106" s="39"/>
@@ -3656,6 +3781,7 @@
       <x:c r="H106" s="36"/>
       <x:c r="I106" s="39"/>
       <x:c r="J106" s="37"/>
+      <x:c r="K106"/>
     </x:row>
     <x:row r="107">
       <x:c r="A107" s="39"/>
@@ -3668,6 +3794,7 @@
       <x:c r="H107" s="36"/>
       <x:c r="I107" s="39"/>
       <x:c r="J107" s="37"/>
+      <x:c r="K107"/>
     </x:row>
     <x:row r="108">
       <x:c r="A108" s="39"/>
@@ -3680,6 +3807,7 @@
       <x:c r="H108" s="36"/>
       <x:c r="I108" s="39"/>
       <x:c r="J108" s="37"/>
+      <x:c r="K108"/>
     </x:row>
     <x:row r="109">
       <x:c r="A109" s="39"/>
@@ -3692,6 +3820,7 @@
       <x:c r="H109" s="36"/>
       <x:c r="I109" s="39"/>
       <x:c r="J109" s="37"/>
+      <x:c r="K109"/>
     </x:row>
     <x:row r="110">
       <x:c r="A110" s="39"/>
@@ -3704,6 +3833,7 @@
       <x:c r="H110" s="36"/>
       <x:c r="I110" s="39"/>
       <x:c r="J110" s="37"/>
+      <x:c r="K110"/>
     </x:row>
     <x:row r="111">
       <x:c r="A111" s="39"/>
@@ -3716,6 +3846,7 @@
       <x:c r="H111" s="36"/>
       <x:c r="I111" s="39"/>
       <x:c r="J111" s="37"/>
+      <x:c r="K111"/>
     </x:row>
     <x:row r="112">
       <x:c r="A112" s="39"/>
@@ -3728,6 +3859,7 @@
       <x:c r="H112" s="36"/>
       <x:c r="I112" s="39"/>
       <x:c r="J112" s="37"/>
+      <x:c r="K112"/>
     </x:row>
     <x:row r="113">
       <x:c r="A113" s="39"/>
@@ -3740,6 +3872,7 @@
       <x:c r="H113" s="36"/>
       <x:c r="I113" s="39"/>
       <x:c r="J113" s="37"/>
+      <x:c r="K113"/>
     </x:row>
     <x:row r="114">
       <x:c r="A114" s="39"/>
@@ -3752,6 +3885,7 @@
       <x:c r="H114" s="36"/>
       <x:c r="I114" s="39"/>
       <x:c r="J114" s="37"/>
+      <x:c r="K114"/>
     </x:row>
     <x:row r="115">
       <x:c r="A115" s="39"/>
@@ -3764,6 +3898,7 @@
       <x:c r="H115" s="36"/>
       <x:c r="I115" s="39"/>
       <x:c r="J115" s="37"/>
+      <x:c r="K115"/>
     </x:row>
     <x:row r="116">
       <x:c r="A116" s="39"/>
@@ -3776,6 +3911,7 @@
       <x:c r="H116" s="36"/>
       <x:c r="I116" s="39"/>
       <x:c r="J116" s="37"/>
+      <x:c r="K116"/>
     </x:row>
     <x:row r="117">
       <x:c r="A117" s="39"/>
@@ -3788,6 +3924,7 @@
       <x:c r="H117" s="36"/>
       <x:c r="I117" s="39"/>
       <x:c r="J117" s="37"/>
+      <x:c r="K117"/>
     </x:row>
     <x:row r="118">
       <x:c r="A118" s="39"/>
@@ -3800,6 +3937,7 @@
       <x:c r="H118" s="36"/>
       <x:c r="I118" s="39"/>
       <x:c r="J118" s="37"/>
+      <x:c r="K118"/>
     </x:row>
     <x:row r="119">
       <x:c r="A119" s="39"/>
@@ -3812,6 +3950,7 @@
       <x:c r="H119" s="36"/>
       <x:c r="I119" s="39"/>
       <x:c r="J119" s="37"/>
+      <x:c r="K119"/>
     </x:row>
     <x:row r="120">
       <x:c r="A120" s="39"/>
@@ -3824,6 +3963,7 @@
       <x:c r="H120" s="36"/>
       <x:c r="I120" s="39"/>
       <x:c r="J120" s="37"/>
+      <x:c r="K120"/>
     </x:row>
     <x:row r="121">
       <x:c r="A121" s="39"/>
@@ -3836,6 +3976,7 @@
       <x:c r="H121" s="36"/>
       <x:c r="I121" s="39"/>
       <x:c r="J121" s="37"/>
+      <x:c r="K121"/>
     </x:row>
     <x:row r="122">
       <x:c r="A122" s="39"/>
@@ -3848,6 +3989,7 @@
       <x:c r="H122" s="36"/>
       <x:c r="I122" s="39"/>
       <x:c r="J122" s="37"/>
+      <x:c r="K122"/>
     </x:row>
     <x:row r="123">
       <x:c r="A123" s="39"/>
@@ -3860,6 +4002,7 @@
       <x:c r="H123" s="36"/>
       <x:c r="I123" s="39"/>
       <x:c r="J123" s="37"/>
+      <x:c r="K123"/>
     </x:row>
     <x:row r="124">
       <x:c r="A124" s="39"/>
@@ -3872,6 +4015,7 @@
       <x:c r="H124" s="36"/>
       <x:c r="I124" s="39"/>
       <x:c r="J124" s="37"/>
+      <x:c r="K124"/>
     </x:row>
     <x:row r="125">
       <x:c r="A125" s="39"/>
@@ -3884,6 +4028,7 @@
       <x:c r="H125" s="36"/>
       <x:c r="I125" s="39"/>
       <x:c r="J125" s="37"/>
+      <x:c r="K125"/>
     </x:row>
     <x:row r="126">
       <x:c r="A126" s="39"/>
@@ -3896,6 +4041,7 @@
       <x:c r="H126" s="36"/>
       <x:c r="I126" s="39"/>
       <x:c r="J126" s="37"/>
+      <x:c r="K126"/>
     </x:row>
     <x:row r="127">
       <x:c r="A127" s="39"/>
@@ -3908,6 +4054,7 @@
       <x:c r="H127" s="36"/>
       <x:c r="I127" s="39"/>
       <x:c r="J127" s="37"/>
+      <x:c r="K127"/>
     </x:row>
     <x:row r="128">
       <x:c r="A128" s="39"/>
@@ -3920,6 +4067,7 @@
       <x:c r="H128" s="36"/>
       <x:c r="I128" s="39"/>
       <x:c r="J128" s="37"/>
+      <x:c r="K128"/>
     </x:row>
     <x:row r="129">
       <x:c r="A129" s="39"/>
@@ -3932,6 +4080,7 @@
       <x:c r="H129" s="36"/>
       <x:c r="I129" s="39"/>
       <x:c r="J129" s="37"/>
+      <x:c r="K129"/>
     </x:row>
     <x:row r="130">
       <x:c r="A130" s="39"/>
@@ -3944,6 +4093,7 @@
       <x:c r="H130" s="36"/>
       <x:c r="I130" s="39"/>
       <x:c r="J130" s="37"/>
+      <x:c r="K130"/>
     </x:row>
     <x:row r="131">
       <x:c r="A131" s="39"/>
@@ -3956,6 +4106,7 @@
       <x:c r="H131" s="36"/>
       <x:c r="I131" s="39"/>
       <x:c r="J131" s="37"/>
+      <x:c r="K131"/>
     </x:row>
     <x:row r="132">
       <x:c r="A132" s="39"/>
@@ -3968,6 +4119,7 @@
       <x:c r="H132" s="36"/>
       <x:c r="I132" s="39"/>
       <x:c r="J132" s="37"/>
+      <x:c r="K132"/>
     </x:row>
     <x:row r="133">
       <x:c r="A133" s="39"/>
@@ -3980,6 +4132,7 @@
       <x:c r="H133" s="36"/>
       <x:c r="I133" s="39"/>
       <x:c r="J133" s="37"/>
+      <x:c r="K133"/>
     </x:row>
     <x:row r="134">
       <x:c r="A134" s="39"/>
@@ -3992,6 +4145,7 @@
       <x:c r="H134" s="36"/>
       <x:c r="I134" s="39"/>
       <x:c r="J134" s="37"/>
+      <x:c r="K134"/>
     </x:row>
     <x:row r="135">
       <x:c r="A135" s="39"/>
@@ -4004,6 +4158,7 @@
       <x:c r="H135" s="36"/>
       <x:c r="I135" s="39"/>
       <x:c r="J135" s="37"/>
+      <x:c r="K135"/>
     </x:row>
     <x:row r="136">
       <x:c r="A136" s="39"/>
@@ -4016,6 +4171,7 @@
       <x:c r="H136" s="36"/>
       <x:c r="I136" s="39"/>
       <x:c r="J136" s="37"/>
+      <x:c r="K136"/>
     </x:row>
     <x:row r="137">
       <x:c r="A137" s="39"/>
@@ -4028,6 +4184,7 @@
       <x:c r="H137" s="36"/>
       <x:c r="I137" s="39"/>
       <x:c r="J137" s="37"/>
+      <x:c r="K137"/>
     </x:row>
     <x:row r="138">
       <x:c r="A138" s="39"/>
@@ -4040,6 +4197,7 @@
       <x:c r="H138" s="36"/>
       <x:c r="I138" s="39"/>
       <x:c r="J138" s="37"/>
+      <x:c r="K138"/>
     </x:row>
     <x:row r="139">
       <x:c r="A139" s="39"/>
@@ -4052,6 +4210,7 @@
       <x:c r="H139" s="36"/>
       <x:c r="I139" s="39"/>
       <x:c r="J139" s="37"/>
+      <x:c r="K139"/>
     </x:row>
     <x:row r="140">
       <x:c r="A140" s="39"/>
@@ -4064,6 +4223,7 @@
       <x:c r="H140" s="36"/>
       <x:c r="I140" s="39"/>
       <x:c r="J140" s="37"/>
+      <x:c r="K140"/>
     </x:row>
     <x:row r="141">
       <x:c r="A141" s="39"/>
@@ -4076,6 +4236,7 @@
       <x:c r="H141" s="36"/>
       <x:c r="I141" s="39"/>
       <x:c r="J141" s="37"/>
+      <x:c r="K141"/>
     </x:row>
     <x:row r="142">
       <x:c r="A142" s="39"/>
@@ -4088,6 +4249,7 @@
       <x:c r="H142" s="36"/>
       <x:c r="I142" s="39"/>
       <x:c r="J142" s="37"/>
+      <x:c r="K142"/>
     </x:row>
     <x:row r="143">
       <x:c r="A143" s="39"/>
@@ -4100,6 +4262,7 @@
       <x:c r="H143" s="36"/>
       <x:c r="I143" s="39"/>
       <x:c r="J143" s="37"/>
+      <x:c r="K143"/>
     </x:row>
     <x:row r="144">
       <x:c r="A144" s="39"/>
@@ -4112,6 +4275,7 @@
       <x:c r="H144" s="36"/>
       <x:c r="I144" s="39"/>
       <x:c r="J144" s="37"/>
+      <x:c r="K144"/>
     </x:row>
     <x:row r="145">
       <x:c r="A145" s="39"/>
@@ -4124,6 +4288,7 @@
       <x:c r="H145" s="36"/>
       <x:c r="I145" s="39"/>
       <x:c r="J145" s="37"/>
+      <x:c r="K145"/>
     </x:row>
     <x:row r="146">
       <x:c r="A146" s="39"/>
@@ -4136,6 +4301,7 @@
       <x:c r="H146" s="36"/>
       <x:c r="I146" s="39"/>
       <x:c r="J146" s="37"/>
+      <x:c r="K146"/>
     </x:row>
     <x:row r="147">
       <x:c r="A147" s="39"/>
@@ -4148,6 +4314,7 @@
       <x:c r="H147" s="36"/>
       <x:c r="I147" s="39"/>
       <x:c r="J147" s="37"/>
+      <x:c r="K147"/>
     </x:row>
     <x:row r="148">
       <x:c r="A148" s="39"/>
@@ -4160,6 +4327,7 @@
       <x:c r="H148" s="36"/>
       <x:c r="I148" s="39"/>
       <x:c r="J148" s="37"/>
+      <x:c r="K148"/>
     </x:row>
     <x:row r="149">
       <x:c r="A149" s="39"/>
@@ -4172,6 +4340,7 @@
       <x:c r="H149" s="36"/>
       <x:c r="I149" s="39"/>
       <x:c r="J149" s="37"/>
+      <x:c r="K149"/>
     </x:row>
     <x:row r="150">
       <x:c r="A150" s="39"/>
@@ -4184,6 +4353,7 @@
       <x:c r="H150" s="36"/>
       <x:c r="I150" s="39"/>
       <x:c r="J150" s="37"/>
+      <x:c r="K150"/>
     </x:row>
     <x:row r="151">
       <x:c r="A151" s="39"/>
@@ -4196,6 +4366,7 @@
       <x:c r="H151" s="36"/>
       <x:c r="I151" s="39"/>
       <x:c r="J151" s="37"/>
+      <x:c r="K151"/>
     </x:row>
     <x:row r="152">
       <x:c r="A152" s="39"/>
@@ -4208,6 +4379,7 @@
       <x:c r="H152" s="36"/>
       <x:c r="I152" s="39"/>
       <x:c r="J152" s="37"/>
+      <x:c r="K152"/>
     </x:row>
     <x:row r="153">
       <x:c r="A153" s="39"/>
@@ -4220,6 +4392,7 @@
       <x:c r="H153" s="36"/>
       <x:c r="I153" s="39"/>
       <x:c r="J153" s="37"/>
+      <x:c r="K153"/>
     </x:row>
     <x:row r="154">
       <x:c r="A154" s="39"/>
@@ -4232,6 +4405,7 @@
       <x:c r="H154" s="36"/>
       <x:c r="I154" s="39"/>
       <x:c r="J154" s="37"/>
+      <x:c r="K154"/>
     </x:row>
     <x:row r="155">
       <x:c r="A155" s="39"/>
@@ -4244,6 +4418,7 @@
       <x:c r="H155" s="36"/>
       <x:c r="I155" s="39"/>
       <x:c r="J155" s="37"/>
+      <x:c r="K155"/>
     </x:row>
     <x:row r="156">
       <x:c r="A156" s="39"/>
@@ -4256,6 +4431,7 @@
       <x:c r="H156" s="36"/>
       <x:c r="I156" s="39"/>
       <x:c r="J156" s="37"/>
+      <x:c r="K156"/>
     </x:row>
     <x:row r="157">
       <x:c r="A157" s="39"/>
@@ -4268,6 +4444,7 @@
       <x:c r="H157" s="36"/>
       <x:c r="I157" s="39"/>
       <x:c r="J157" s="37"/>
+      <x:c r="K157"/>
     </x:row>
     <x:row r="158">
       <x:c r="A158" s="39"/>
@@ -4280,6 +4457,7 @@
       <x:c r="H158" s="36"/>
       <x:c r="I158" s="39"/>
       <x:c r="J158" s="37"/>
+      <x:c r="K158"/>
     </x:row>
     <x:row r="159">
       <x:c r="A159" s="39"/>
@@ -4292,6 +4470,7 @@
       <x:c r="H159" s="36"/>
       <x:c r="I159" s="39"/>
       <x:c r="J159" s="37"/>
+      <x:c r="K159"/>
     </x:row>
     <x:row r="160">
       <x:c r="A160" s="39"/>
@@ -4304,6 +4483,7 @@
       <x:c r="H160" s="36"/>
       <x:c r="I160" s="39"/>
       <x:c r="J160" s="37"/>
+      <x:c r="K160"/>
     </x:row>
     <x:row r="161">
       <x:c r="A161" s="39"/>
@@ -4316,6 +4496,7 @@
       <x:c r="H161" s="36"/>
       <x:c r="I161" s="39"/>
       <x:c r="J161" s="37"/>
+      <x:c r="K161"/>
     </x:row>
     <x:row r="162">
       <x:c r="A162" s="39"/>
@@ -4328,6 +4509,7 @@
       <x:c r="H162" s="36"/>
       <x:c r="I162" s="39"/>
       <x:c r="J162" s="37"/>
+      <x:c r="K162"/>
     </x:row>
     <x:row r="163">
       <x:c r="A163" s="39"/>
@@ -4340,6 +4522,7 @@
       <x:c r="H163" s="36"/>
       <x:c r="I163" s="39"/>
       <x:c r="J163" s="37"/>
+      <x:c r="K163"/>
     </x:row>
     <x:row r="164">
       <x:c r="A164" s="39"/>
@@ -4352,6 +4535,7 @@
       <x:c r="H164" s="36"/>
       <x:c r="I164" s="39"/>
       <x:c r="J164" s="37"/>
+      <x:c r="K164"/>
     </x:row>
     <x:row r="165">
       <x:c r="A165" s="39"/>
@@ -4364,6 +4548,7 @@
       <x:c r="H165" s="36"/>
       <x:c r="I165" s="39"/>
       <x:c r="J165" s="37"/>
+      <x:c r="K165"/>
     </x:row>
     <x:row r="166">
       <x:c r="A166" s="39"/>
@@ -4376,6 +4561,7 @@
       <x:c r="H166" s="36"/>
       <x:c r="I166" s="39"/>
       <x:c r="J166" s="37"/>
+      <x:c r="K166"/>
     </x:row>
     <x:row r="167">
       <x:c r="A167" s="39"/>
@@ -4388,6 +4574,7 @@
       <x:c r="H167" s="36"/>
       <x:c r="I167" s="39"/>
       <x:c r="J167" s="37"/>
+      <x:c r="K167"/>
     </x:row>
     <x:row r="168">
       <x:c r="A168" s="39"/>
@@ -4400,6 +4587,7 @@
       <x:c r="H168" s="36"/>
       <x:c r="I168" s="39"/>
       <x:c r="J168" s="37"/>
+      <x:c r="K168"/>
     </x:row>
     <x:row r="169">
       <x:c r="A169" s="39"/>
@@ -4412,6 +4600,7 @@
       <x:c r="H169" s="36"/>
       <x:c r="I169" s="39"/>
       <x:c r="J169" s="37"/>
+      <x:c r="K169"/>
     </x:row>
     <x:row r="170">
       <x:c r="A170" s="39"/>
@@ -4424,6 +4613,7 @@
       <x:c r="H170" s="36"/>
       <x:c r="I170" s="39"/>
       <x:c r="J170" s="37"/>
+      <x:c r="K170"/>
     </x:row>
     <x:row r="171">
       <x:c r="A171" s="39"/>
@@ -4436,6 +4626,7 @@
       <x:c r="H171" s="36"/>
       <x:c r="I171" s="39"/>
       <x:c r="J171" s="37"/>
+      <x:c r="K171"/>
     </x:row>
     <x:row r="172">
       <x:c r="A172" s="39"/>
@@ -4448,6 +4639,7 @@
       <x:c r="H172" s="36"/>
       <x:c r="I172" s="39"/>
       <x:c r="J172" s="37"/>
+      <x:c r="K172"/>
     </x:row>
     <x:row r="173">
       <x:c r="A173" s="39"/>
@@ -4460,6 +4652,7 @@
       <x:c r="H173" s="36"/>
       <x:c r="I173" s="39"/>
       <x:c r="J173" s="37"/>
+      <x:c r="K173"/>
     </x:row>
     <x:row r="174">
       <x:c r="A174" s="39"/>
@@ -4472,6 +4665,7 @@
       <x:c r="H174" s="36"/>
       <x:c r="I174" s="39"/>
       <x:c r="J174" s="37"/>
+      <x:c r="K174"/>
     </x:row>
     <x:row r="175">
       <x:c r="A175" s="39"/>
@@ -4484,6 +4678,7 @@
       <x:c r="H175" s="36"/>
       <x:c r="I175" s="39"/>
       <x:c r="J175" s="37"/>
+      <x:c r="K175"/>
     </x:row>
     <x:row r="176">
       <x:c r="A176" s="39"/>
@@ -4496,6 +4691,7 @@
       <x:c r="H176" s="36"/>
       <x:c r="I176" s="39"/>
       <x:c r="J176" s="37"/>
+      <x:c r="K176"/>
     </x:row>
     <x:row r="177">
       <x:c r="A177" s="39"/>
@@ -4508,6 +4704,7 @@
       <x:c r="H177" s="36"/>
       <x:c r="I177" s="39"/>
       <x:c r="J177" s="37"/>
+      <x:c r="K177"/>
     </x:row>
     <x:row r="178">
       <x:c r="A178" s="39"/>
@@ -4520,6 +4717,7 @@
       <x:c r="H178" s="36"/>
       <x:c r="I178" s="39"/>
       <x:c r="J178" s="37"/>
+      <x:c r="K178"/>
     </x:row>
     <x:row r="179">
       <x:c r="A179" s="39"/>
@@ -4532,6 +4730,7 @@
       <x:c r="H179" s="36"/>
       <x:c r="I179" s="39"/>
       <x:c r="J179" s="37"/>
+      <x:c r="K179"/>
     </x:row>
     <x:row r="180">
       <x:c r="A180" s="39"/>
@@ -4544,6 +4743,7 @@
       <x:c r="H180" s="36"/>
       <x:c r="I180" s="39"/>
       <x:c r="J180" s="37"/>
+      <x:c r="K180"/>
     </x:row>
     <x:row r="181">
       <x:c r="A181" s="39"/>
@@ -4556,6 +4756,7 @@
       <x:c r="H181" s="36"/>
       <x:c r="I181" s="39"/>
       <x:c r="J181" s="37"/>
+      <x:c r="K181"/>
     </x:row>
     <x:row r="182">
       <x:c r="A182" s="39"/>
@@ -4568,6 +4769,7 @@
       <x:c r="H182" s="36"/>
       <x:c r="I182" s="39"/>
       <x:c r="J182" s="37"/>
+      <x:c r="K182"/>
     </x:row>
     <x:row r="183">
       <x:c r="A183" s="39"/>
@@ -4580,6 +4782,7 @@
       <x:c r="H183" s="36"/>
       <x:c r="I183" s="39"/>
       <x:c r="J183" s="37"/>
+      <x:c r="K183"/>
     </x:row>
     <x:row r="184">
       <x:c r="A184" s="39"/>
@@ -4592,6 +4795,7 @@
       <x:c r="H184" s="36"/>
       <x:c r="I184" s="39"/>
       <x:c r="J184" s="37"/>
+      <x:c r="K184"/>
     </x:row>
     <x:row r="185">
       <x:c r="A185" s="39"/>
@@ -4604,6 +4808,7 @@
       <x:c r="H185" s="36"/>
       <x:c r="I185" s="39"/>
       <x:c r="J185" s="37"/>
+      <x:c r="K185"/>
     </x:row>
     <x:row r="186">
       <x:c r="A186" s="39"/>
@@ -4616,6 +4821,7 @@
       <x:c r="H186" s="36"/>
       <x:c r="I186" s="39"/>
       <x:c r="J186" s="37"/>
+      <x:c r="K186"/>
     </x:row>
     <x:row r="187">
       <x:c r="A187" s="39"/>
@@ -4628,6 +4834,7 @@
       <x:c r="H187" s="36"/>
       <x:c r="I187" s="39"/>
       <x:c r="J187" s="37"/>
+      <x:c r="K187"/>
     </x:row>
     <x:row r="188">
       <x:c r="A188" s="39"/>
@@ -4640,6 +4847,7 @@
       <x:c r="H188" s="36"/>
       <x:c r="I188" s="39"/>
       <x:c r="J188" s="37"/>
+      <x:c r="K188"/>
     </x:row>
     <x:row r="189">
       <x:c r="A189" s="39"/>
@@ -4652,6 +4860,7 @@
       <x:c r="H189" s="36"/>
       <x:c r="I189" s="39"/>
       <x:c r="J189" s="37"/>
+      <x:c r="K189"/>
     </x:row>
     <x:row r="190">
       <x:c r="A190" s="39"/>
@@ -4664,6 +4873,7 @@
       <x:c r="H190" s="36"/>
       <x:c r="I190" s="39"/>
       <x:c r="J190" s="37"/>
+      <x:c r="K190"/>
     </x:row>
     <x:row r="191">
       <x:c r="A191" s="39"/>
@@ -4676,6 +4886,7 @@
       <x:c r="H191" s="36"/>
       <x:c r="I191" s="39"/>
       <x:c r="J191" s="37"/>
+      <x:c r="K191"/>
     </x:row>
     <x:row r="192">
       <x:c r="A192" s="39"/>
@@ -4688,6 +4899,7 @@
       <x:c r="H192" s="36"/>
       <x:c r="I192" s="39"/>
       <x:c r="J192" s="37"/>
+      <x:c r="K192"/>
     </x:row>
     <x:row r="193">
       <x:c r="A193" s="39"/>
@@ -4700,6 +4912,7 @@
       <x:c r="H193" s="36"/>
       <x:c r="I193" s="39"/>
       <x:c r="J193" s="37"/>
+      <x:c r="K193"/>
     </x:row>
     <x:row r="194">
       <x:c r="A194" s="39"/>
@@ -4712,6 +4925,7 @@
       <x:c r="H194" s="36"/>
       <x:c r="I194" s="39"/>
       <x:c r="J194" s="37"/>
+      <x:c r="K194"/>
     </x:row>
     <x:row r="195">
       <x:c r="A195" s="39"/>
@@ -4724,6 +4938,7 @@
       <x:c r="H195" s="36"/>
       <x:c r="I195" s="39"/>
       <x:c r="J195" s="37"/>
+      <x:c r="K195"/>
     </x:row>
     <x:row r="196">
       <x:c r="A196" s="39"/>
@@ -4736,6 +4951,7 @@
       <x:c r="H196" s="36"/>
       <x:c r="I196" s="39"/>
       <x:c r="J196" s="37"/>
+      <x:c r="K196"/>
     </x:row>
     <x:row r="197">
       <x:c r="A197" s="39"/>
@@ -4748,6 +4964,7 @@
       <x:c r="H197" s="36"/>
       <x:c r="I197" s="39"/>
       <x:c r="J197" s="37"/>
+      <x:c r="K197"/>
     </x:row>
     <x:row r="198">
       <x:c r="A198" s="39"/>
@@ -4760,6 +4977,7 @@
       <x:c r="H198" s="36"/>
       <x:c r="I198" s="39"/>
       <x:c r="J198" s="37"/>
+      <x:c r="K198"/>
     </x:row>
     <x:row r="199">
       <x:c r="A199" s="39"/>
@@ -4772,6 +4990,7 @@
       <x:c r="H199" s="36"/>
       <x:c r="I199" s="39"/>
       <x:c r="J199" s="37"/>
+      <x:c r="K199"/>
     </x:row>
     <x:row r="200">
       <x:c r="A200" s="39"/>
@@ -4784,6 +5003,7 @@
       <x:c r="H200" s="36"/>
       <x:c r="I200" s="39"/>
       <x:c r="J200" s="37"/>
+      <x:c r="K200"/>
     </x:row>
     <x:row r="201">
       <x:c r="A201" s="39"/>
@@ -4796,6 +5016,7 @@
       <x:c r="H201" s="36"/>
       <x:c r="I201" s="39"/>
       <x:c r="J201" s="37"/>
+      <x:c r="K201"/>
     </x:row>
     <x:row r="204">
       <x:c r="A204" s="43" t="str">
@@ -4860,7 +5081,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R11a97a59062c4527"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rec8e871fa15a4dc5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>